<commit_message>
making file with combined app.tech reductions
</commit_message>
<xml_diff>
--- a/reductions/data/data_2014.xlsx
+++ b/reductions/data/data_2014.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au583430_uni_au_dk/Documents/Documents/GitHub/GD-NH3/reductions/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="8_{5E20B5B0-32C7-431D-8683-E50ABE62E15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{173BE45A-32F3-49DE-B437-2D8E3D0E1C01}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{5E20B5B0-32C7-431D-8683-E50ABE62E15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FB600B0-F8B8-480D-890A-DB8F720901AF}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-45" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{7C63DCD4-7913-4208-A171-6214FA8E3972}"/>
+    <workbookView xWindow="1485" yWindow="2580" windowWidth="21600" windowHeight="10935" activeTab="1" xr2:uid="{7C63DCD4-7913-4208-A171-6214FA8E3972}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="21">
   <si>
     <t>grass</t>
   </si>
@@ -160,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -172,6 +172,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -699,187 +702,147 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E141CA5-1FB4-4DAD-BBC1-66FB61386D09}">
-  <dimension ref="A1:F1048570"/>
+  <dimension ref="A1:E1048567"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4">
+        <f>data!C2+data!C3</f>
+        <v>10</v>
+      </c>
+      <c r="C2" s="4">
+        <f>(data!C2*data!D2+data!C3*data!D3)/(data!C2+data!C3)</f>
+        <v>75</v>
+      </c>
+      <c r="D2" s="4">
+        <f>data!E3</f>
+        <v>23</v>
+      </c>
+      <c r="E2" s="4">
+        <f>data!F2</f>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4">
+        <f>data!C4</f>
+        <v>2</v>
+      </c>
+      <c r="C3" s="4">
+        <f>data!D4</f>
+        <v>95</v>
+      </c>
+      <c r="D3" s="4">
+        <f>data!E4</f>
+        <v>95</v>
+      </c>
+      <c r="E3" s="4">
+        <f>data!F4</f>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="4">
+        <f>data!C5+data!C6</f>
+        <v>4</v>
+      </c>
+      <c r="C4" s="4">
+        <f>(data!C5*data!D5+data!C6*data!D6)/(data!C5+data!C6)</f>
+        <v>64</v>
+      </c>
+      <c r="D4" s="4">
+        <f>data!E6</f>
+        <v>38</v>
+      </c>
+      <c r="E4" s="4">
+        <f>data!F6</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="4">
+        <f>data!C7+data!C8</f>
+        <v>12</v>
+      </c>
+      <c r="C5" s="5">
+        <f>(data!C7*data!D7+data!C8*data!D8)/(data!C7+data!C8)</f>
+        <v>36.166666666666664</v>
+      </c>
+      <c r="D5" s="4">
+        <f>data!E8</f>
         <v>0</v>
       </c>
-      <c r="C2" s="4">
-        <v>5</v>
-      </c>
-      <c r="D2" s="4">
-        <v>80</v>
-      </c>
-      <c r="E2" s="4">
-        <v>60</v>
-      </c>
-      <c r="F2" s="4">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="4">
-        <v>5</v>
-      </c>
-      <c r="D3" s="4">
-        <v>70</v>
-      </c>
-      <c r="E3" s="4">
-        <v>23</v>
-      </c>
-      <c r="F3" s="4">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="4">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4">
-        <v>95</v>
-      </c>
-      <c r="E4" s="4">
-        <v>95</v>
-      </c>
-      <c r="F4" s="4">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="4">
-        <v>2</v>
-      </c>
-      <c r="D5" s="4">
-        <v>64</v>
-      </c>
       <c r="E5" s="4">
-        <v>57</v>
-      </c>
-      <c r="F5" s="4">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="4">
-        <v>2</v>
-      </c>
-      <c r="D6" s="4">
-        <v>64</v>
-      </c>
-      <c r="E6" s="4">
-        <v>38</v>
-      </c>
-      <c r="F6" s="4">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C7" s="4">
-        <v>5</v>
-      </c>
-      <c r="D7" s="4">
-        <v>35</v>
-      </c>
-      <c r="E7" s="4">
-        <v>0</v>
-      </c>
-      <c r="F7" s="4">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="4">
-        <v>7</v>
-      </c>
-      <c r="D8" s="4">
-        <v>37</v>
-      </c>
-      <c r="E8" s="4">
-        <v>0</v>
-      </c>
-      <c r="F8" s="4">
+        <f>data!F8</f>
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D11" s="4"/>
-    </row>
-    <row r="1048570" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1048570" s="1"/>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C7" s="4"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+    </row>
+    <row r="1048567" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1048567" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>